<commit_message>
Fix dashboard headers and cumulative data logic
</commit_message>
<xml_diff>
--- a/data/monthly_report_2026-02.xlsx
+++ b/data/monthly_report_2026-02.xlsx
@@ -431,7 +431,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>market</t>
+          <t>시장구분</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -441,57 +441,57 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>종목명</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>현재가</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>foreign_rate</t>
+          <t>현재_외국인비중</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>prev_close</t>
+          <t>어제_종가</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>prev_foreign_rate</t>
+          <t>어제_외국인비중</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>change_rate</t>
+          <t>등락률</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>recent_posts_count</t>
+          <t>당일_게시글수</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>posts_summary</t>
+          <t>게시물_요약</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>sentiment</t>
+          <t>감정분석</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>top_keywords</t>
+          <t>Top_Keyword</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>is_last_captured</t>
+          <t>연속_등록</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">

</xml_diff>